<commit_message>
Stabilize import flow and platform UI
</commit_message>
<xml_diff>
--- a/templates/用例集导入模板.xlsx
+++ b/templates/用例集导入模板.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ROG\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ROG\Desktop\TestChamberV7\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8D8C3F-16EF-4111-9064-ED9CB338AA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EA03C3-005D-4E7B-8BE0-2965E1808525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,6 +72,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
@@ -126,10 +134,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>